<commit_message>
Workbooks: strip ghost cell borders left by the Reasons rebuild
The June-1 sweep rewrote row values and copied donor styles, but cells
whose donor had no explicit style kept the OLD row's formatting — so
the retired layout's dated-line underlines showed up under formation
and season rows (e.g. Fixtures/Laptop/Priya in 32-1's facsimile).
Cleared borders on every non-Balance row in the rebuilt regions
(ruled lines on Balance rows preserved: 18/18 in the extraction, 0
ghosts, was 3), recomputed cached values, regenerated the steps JS —
all 20 extraction invariants pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
+++ b/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
@@ -74,7 +74,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -102,11 +102,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,6 +139,8 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1836,7 +1839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="B1:D60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1907,7 +1910,7 @@
           <t>Fixtures — Company received at formation (June 1)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n"/>
+      <c r="C7" s="22" t="n"/>
       <c r="D7" s="4" t="n">
         <v>750</v>
       </c>

</xml_diff>

<commit_message>
Workbooks: rebuild Reasons outline groups after the June-1 restructure
The sweep moved row content but left row-level outline metadata
(outlineLevel/hidden/collapsed) at old positions — [+] toggles landed on
arbitrary rows and most of the tab was hidden. Regrouped rule-based per
the original design (summaryBelow: item runs level-1 hidden, the dated
Balance line below each run is the collapsed summary) across the ten
Reasons sheets, 4-1 Working Tab, and Members-Capital step 0; recached,
regenerated; 20/20 invariants; 32-1 Reasons browser-verified.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
+++ b/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
@@ -1864,7 +1864,7 @@
       <c r="C2" s="11" t="n"/>
       <c r="D2" s="11" t="n"/>
     </row>
-    <row r="3" outlineLevel="1">
+    <row r="3" hidden="1" outlineLevel="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Cash — Company received at formation (June 1)</t>
@@ -1874,7 +1874,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="4" outlineLevel="1">
+    <row r="4" hidden="1" outlineLevel="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Right of Use — Company received at formation (June 1)</t>
@@ -1884,7 +1884,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="5" outlineLevel="1">
+    <row r="5" hidden="1" outlineLevel="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Parts — Company received at formation (June 1)</t>
@@ -1894,7 +1894,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" outlineLevel="1">
+    <row r="6" hidden="1" outlineLevel="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Tools &amp; Repair Equipment — Company received at formation (June 1)</t>
@@ -1904,7 +1904,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="1" outlineLevel="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Fixtures — Company received at formation (June 1)</t>
@@ -1915,7 +1915,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="1" outlineLevel="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Laptop — Company received at formation (June 1)</t>
@@ -1925,7 +1925,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="1" outlineLevel="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Credit Card — Company assumed the claim at formation (June 1)</t>
@@ -1936,7 +1936,7 @@
         <v>-2030</v>
       </c>
     </row>
-    <row r="10" outlineLevel="1">
+    <row r="10" hidden="1" outlineLevel="1">
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Customer Deposit — Company assumed the claim at formation (June 1)</t>
@@ -1946,7 +1946,7 @@
         <v>-220</v>
       </c>
     </row>
-    <row r="11" outlineLevel="1">
+    <row r="11" collapsed="1">
       <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Balance, August 31, 2026</t>
@@ -1959,11 +1959,11 @@
         <v/>
       </c>
     </row>
-    <row r="12" outlineLevel="1">
+    <row r="12">
       <c r="B12" s="3" t="n"/>
       <c r="D12" s="4" t="n"/>
     </row>
-    <row r="13" outlineLevel="1">
+    <row r="13">
       <c r="B13" s="6" t="inlineStr">
         <is>
           <t>GENERATED</t>
@@ -1972,7 +1972,7 @@
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="11" t="n"/>
     </row>
-    <row r="14" outlineLevel="1">
+    <row r="14" hidden="1" outlineLevel="1">
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Dana R.</t>
@@ -1982,7 +1982,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" outlineLevel="1">
+    <row r="15" hidden="1" outlineLevel="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Parts used — Dana R.</t>
@@ -1992,7 +1992,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="16" outlineLevel="1">
+    <row r="16" hidden="1" outlineLevel="1">
       <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Marcus T.</t>
@@ -2002,7 +2002,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="17" outlineLevel="1">
+    <row r="17" hidden="1" outlineLevel="1">
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Priya S.</t>
@@ -2012,7 +2012,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="18" outlineLevel="1">
+    <row r="18" hidden="1" outlineLevel="1">
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Parts used — Priya S.</t>
@@ -2022,7 +2022,7 @@
         <v>-25</v>
       </c>
     </row>
-    <row r="19" outlineLevel="1">
+    <row r="19" hidden="1" outlineLevel="1">
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Liam O.</t>
@@ -2032,7 +2032,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="20" outlineLevel="1">
+    <row r="20" hidden="1" outlineLevel="1">
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Parts used — Liam O.</t>
@@ -2042,7 +2042,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="21" outlineLevel="1">
+    <row r="21" hidden="1" outlineLevel="1">
       <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Sofia M.</t>
@@ -2052,7 +2052,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="22" outlineLevel="1">
+    <row r="22" hidden="1" outlineLevel="1">
       <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Jamal W.</t>
@@ -2062,7 +2062,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="23" outlineLevel="1">
+    <row r="23" hidden="1" outlineLevel="1">
       <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Parts used — Jamal W.</t>
@@ -2072,7 +2072,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="24" outlineLevel="1">
+    <row r="24" hidden="1" outlineLevel="1">
       <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Erin K.</t>
@@ -2082,7 +2082,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="25" outlineLevel="1">
+    <row r="25" hidden="1" outlineLevel="1">
       <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Parts used — Erin K.</t>
@@ -2092,7 +2092,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="26" outlineLevel="1">
+    <row r="26" hidden="1" outlineLevel="1">
       <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Noah B.</t>
@@ -2102,7 +2102,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="27" outlineLevel="1">
+    <row r="27" hidden="1" outlineLevel="1">
       <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Parts used — Noah B.</t>
@@ -2112,7 +2112,7 @@
         <v>-65</v>
       </c>
     </row>
-    <row r="28" outlineLevel="1">
+    <row r="28" hidden="1" outlineLevel="1">
       <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Rent used — June</t>
@@ -2122,7 +2122,7 @@
         <v>-650</v>
       </c>
     </row>
-    <row r="29" outlineLevel="1">
+    <row r="29" hidden="1" outlineLevel="1">
       <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Rent used — July</t>
@@ -2132,7 +2132,7 @@
         <v>-650</v>
       </c>
     </row>
-    <row r="30" outlineLevel="1">
+    <row r="30" hidden="1" outlineLevel="1">
       <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Grace L.</t>
@@ -2142,7 +2142,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="31" outlineLevel="1">
+    <row r="31" hidden="1" outlineLevel="1">
       <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Parts used — Grace L.</t>
@@ -2152,7 +2152,7 @@
         <v>-35</v>
       </c>
     </row>
-    <row r="32" outlineLevel="1">
+    <row r="32" hidden="1" outlineLevel="1">
       <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Theo H.</t>
@@ -2162,7 +2162,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="33" outlineLevel="1">
+    <row r="33" hidden="1" outlineLevel="1">
       <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Parts used — Theo H.</t>
@@ -2172,7 +2172,7 @@
         <v>-25</v>
       </c>
     </row>
-    <row r="34" outlineLevel="1">
+    <row r="34" hidden="1" outlineLevel="1">
       <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Maya P.</t>
@@ -2182,7 +2182,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="35" outlineLevel="1">
+    <row r="35" hidden="1" outlineLevel="1">
       <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Parts used — Maya P.</t>
@@ -2192,7 +2192,7 @@
         <v>-125</v>
       </c>
     </row>
-    <row r="36" outlineLevel="1">
+    <row r="36" hidden="1" outlineLevel="1">
       <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Owen C.</t>
@@ -2202,7 +2202,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="37" outlineLevel="1">
+    <row r="37" hidden="1" outlineLevel="1">
       <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Parts used — Owen C.</t>
@@ -2212,7 +2212,7 @@
         <v>-55</v>
       </c>
     </row>
-    <row r="38" outlineLevel="1">
+    <row r="38" hidden="1" outlineLevel="1">
       <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Ava D.</t>
@@ -2222,7 +2222,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="39" outlineLevel="1">
+    <row r="39" hidden="1" outlineLevel="1">
       <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Parts used — Ava D.</t>
@@ -2232,7 +2232,7 @@
         <v>-45</v>
       </c>
     </row>
-    <row r="40" outlineLevel="1">
+    <row r="40" hidden="1" outlineLevel="1">
       <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Leo F.</t>
@@ -2242,7 +2242,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="41" outlineLevel="1">
+    <row r="41" hidden="1" outlineLevel="1">
       <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Parts used — Leo F.</t>
@@ -2252,7 +2252,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="42" outlineLevel="1">
+    <row r="42" hidden="1" outlineLevel="1">
       <c r="B42" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Nina V.</t>
@@ -2262,7 +2262,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="43" outlineLevel="1">
+    <row r="43" hidden="1" outlineLevel="1">
       <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Parts used — Nina V.</t>
@@ -2272,7 +2272,7 @@
         <v>-80</v>
       </c>
     </row>
-    <row r="44" outlineLevel="1">
+    <row r="44" hidden="1" outlineLevel="1">
       <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Rent used — August</t>
@@ -2282,7 +2282,7 @@
         <v>-650</v>
       </c>
     </row>
-    <row r="45" outlineLevel="1">
+    <row r="45" hidden="1" outlineLevel="1">
       <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Caleb G.</t>
@@ -2292,7 +2292,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="46" outlineLevel="1">
+    <row r="46" hidden="1" outlineLevel="1">
       <c r="B46" s="3" t="inlineStr">
         <is>
           <t>Parts used — Caleb G.</t>
@@ -2302,7 +2302,7 @@
         <v>-25</v>
       </c>
     </row>
-    <row r="47" outlineLevel="1">
+    <row r="47" hidden="1" outlineLevel="1">
       <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Ruth A.</t>
@@ -2312,7 +2312,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="48" outlineLevel="1">
+    <row r="48" hidden="1" outlineLevel="1">
       <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Parts used — Ruth A.</t>
@@ -2322,7 +2322,7 @@
         <v>-129</v>
       </c>
     </row>
-    <row r="49" outlineLevel="1">
+    <row r="49" hidden="1" outlineLevel="1">
       <c r="B49" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Sam Q.</t>
@@ -2332,7 +2332,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="50" outlineLevel="1">
+    <row r="50" hidden="1" outlineLevel="1">
       <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Parts used — Sam Q.</t>
@@ -2342,7 +2342,7 @@
         <v>-70</v>
       </c>
     </row>
-    <row r="51" outlineLevel="1">
+    <row r="51" hidden="1" outlineLevel="1">
       <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Repair collected — Westville Bike Share</t>
@@ -2352,7 +2352,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="52" outlineLevel="1">
+    <row r="52" hidden="1" outlineLevel="1">
       <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Parts used — Westville Bike Share</t>
@@ -2362,7 +2362,7 @@
         <v>-105</v>
       </c>
     </row>
-    <row r="53" outlineLevel="1">
+    <row r="53" hidden="1" outlineLevel="1">
       <c r="B53" s="3" t="inlineStr">
         <is>
           <t>Parts used — Ridgeline Trail Crew</t>
@@ -2372,7 +2372,7 @@
         <v>-75</v>
       </c>
     </row>
-    <row r="54" outlineLevel="1">
+    <row r="54" hidden="1" outlineLevel="1">
       <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Frame delivered — J. Smith (deposit earned)</t>
@@ -2382,7 +2382,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="55" outlineLevel="1">
+    <row r="55" hidden="1" outlineLevel="1">
       <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Parts used — J. Smith</t>
@@ -2392,7 +2392,7 @@
         <v>-36</v>
       </c>
     </row>
-    <row r="56" outlineLevel="1">
+    <row r="56" collapsed="1">
       <c r="B56" s="16" t="inlineStr">
         <is>
           <t>Balance, August 31, 2026</t>
@@ -2405,11 +2405,11 @@
         <v/>
       </c>
     </row>
-    <row r="57" outlineLevel="1">
+    <row r="57">
       <c r="B57" s="3" t="n"/>
       <c r="D57" s="4" t="n"/>
     </row>
-    <row r="58" outlineLevel="1">
+    <row r="58">
       <c r="B58" s="6" t="inlineStr">
         <is>
           <t>WITHDRAWN</t>
@@ -2418,7 +2418,7 @@
       <c r="C58" s="11" t="n"/>
       <c r="D58" s="11" t="n"/>
     </row>
-    <row r="59" outlineLevel="1">
+    <row r="59" hidden="1" outlineLevel="1">
       <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Owner's draw — money taken out for personal use</t>
@@ -2428,7 +2428,7 @@
         <v>-600</v>
       </c>
     </row>
-    <row r="60" outlineLevel="1">
+    <row r="60" collapsed="1">
       <c r="B60" s="16" t="inlineStr">
         <is>
           <t>Balance, August 31, 2026</t>

</xml_diff>

<commit_message>
Workbooks: asset/liability ledgers open at formation (ruling 17, cont'd)
Rick's click-through caught the remaining boundary violation: the
Company's Assets/Liabilities ledgers still opened with the member's May
personal history (the lease, 'Repair, customer paid' rows, 'Covered
from your personal funds', card charge history). Each ledger's pre-June
segment is now a single formation row — 'Company received at formation
(June 1)' / 'Company assumed the claim at formation (June 1)' — with
season activity unchanged, across all ten workbooks (Beg's continuous-
run layout handled separately; Accounts Receivable sections rewired).
Outline groups rebuilt for the ledger sheets; extractor's cash anchor
moved to the formation label; recached; regenerated; 20/20 invariants;
32-1 Assets/Reasons browser-verified.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
+++ b/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D120"/>
+  <dimension ref="B1:D88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -535,157 +535,157 @@
     <row r="3" hidden="1" outlineLevel="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Rent paid in advance (the lease)</t>
+          <t>Company received at formation (June 1)</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-1300</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="4" hidden="1" outlineLevel="1">
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Park Tool repair stand</t>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Dana R.</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>-200</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" hidden="1" outlineLevel="1">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Repair, customer paid</t>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Marcus T.</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>340</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" hidden="1" outlineLevel="1">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Repair, customer paid</t>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Priya S.</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>180</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" hidden="1" outlineLevel="1">
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Repair, customer paid</t>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Liam O.</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>80</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" hidden="1" outlineLevel="1">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Repair, customer paid</t>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Sofia M.</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" hidden="1" outlineLevel="1">
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Repair, customer paid</t>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Jamal W.</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>130</v>
+        <v>360</v>
       </c>
     </row>
     <row r="10" hidden="1" outlineLevel="1">
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Smith's deposit received</t>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Erin K.</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="11" hidden="1" outlineLevel="1">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Repair, customer paid</t>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Noah B.</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>100</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" hidden="1" outlineLevel="1">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Repair, customer paid</t>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Grace L.</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" hidden="1" outlineLevel="1">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Covered from your personal funds</t>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Theo H.</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>160</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" hidden="1" outlineLevel="1">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Deposited to open the LLC bank account</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>1300</v>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Repair collected — Maya P.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Dana R.</t>
+          <t>Repair collected — Owen C.</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>120</v>
+        <v>360</v>
       </c>
     </row>
     <row r="16" hidden="1" outlineLevel="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Marcus T.</t>
+          <t>Repair collected — Ava D.</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>150</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" hidden="1" outlineLevel="1">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Priya S.</t>
+          <t>Repair collected — Leo F.</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>270</v>
+        <v>240</v>
       </c>
     </row>
     <row r="18" hidden="1" outlineLevel="1">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Liam O.</t>
+          <t>Repair collected — Nina V.</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
@@ -695,341 +695,357 @@
     <row r="19" hidden="1" outlineLevel="1">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Sofia M.</t>
+          <t>Repair collected — Caleb G.</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20" hidden="1" outlineLevel="1">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Jamal W.</t>
+          <t>Repair collected — Ruth A.</t>
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>360</v>
+        <v>485</v>
       </c>
     </row>
     <row r="21" hidden="1" outlineLevel="1">
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Erin K.</t>
+          <t>Repair collected — Sam Q.</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>225</v>
+        <v>390</v>
       </c>
     </row>
     <row r="22" hidden="1" outlineLevel="1">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Noah B.</t>
+          <t>Repair collected — Westville Bike Share</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>210</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23" hidden="1" outlineLevel="1">
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Grace L.</t>
+          <t>Parts bought — June</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>240</v>
+        <v>-500</v>
       </c>
     </row>
     <row r="24" hidden="1" outlineLevel="1">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Theo H.</t>
+          <t>Parts bought — July</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>240</v>
+        <v>-400</v>
       </c>
     </row>
     <row r="25" hidden="1" outlineLevel="1">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Maya P.</t>
+          <t>Parts bought — August</t>
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>450</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="26" hidden="1" outlineLevel="1">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Owen C.</t>
+          <t>Rent paid — June</t>
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>360</v>
+        <v>-650</v>
       </c>
     </row>
     <row r="27" hidden="1" outlineLevel="1">
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Ava D.</t>
+          <t>Rent paid — July</t>
         </is>
       </c>
       <c r="D27" s="4" t="n">
-        <v>270</v>
+        <v>-650</v>
       </c>
     </row>
     <row r="28" hidden="1" outlineLevel="1">
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Leo F.</t>
+          <t>Rent paid — August</t>
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>240</v>
+        <v>-650</v>
       </c>
     </row>
     <row r="29" hidden="1" outlineLevel="1">
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Nina V.</t>
+          <t>New repair tool</t>
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>300</v>
+        <v>-400</v>
       </c>
     </row>
     <row r="30" hidden="1" outlineLevel="1">
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Caleb G.</t>
+          <t>Credit card paid off</t>
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>240</v>
+        <v>-2030</v>
       </c>
     </row>
     <row r="31" hidden="1" outlineLevel="1">
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Repair collected — Ruth A.</t>
+          <t>Money taken out for personal use</t>
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="32" hidden="1" outlineLevel="1">
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Repair collected — Sam Q.</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="33" hidden="1" outlineLevel="1">
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Repair collected — Westville Bike Share</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="34" hidden="1" outlineLevel="1">
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Parts bought — June</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="n">
-        <v>-500</v>
-      </c>
-    </row>
-    <row r="35" hidden="1" outlineLevel="1">
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Parts bought — July</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="n">
-        <v>-400</v>
-      </c>
-    </row>
-    <row r="36" hidden="1" outlineLevel="1">
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>Parts bought — August</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>-300</v>
-      </c>
-    </row>
-    <row r="37" hidden="1" outlineLevel="1">
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Rent paid — June</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>-650</v>
-      </c>
-    </row>
-    <row r="38" hidden="1" outlineLevel="1">
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Rent paid — July</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="n">
-        <v>-650</v>
-      </c>
-    </row>
-    <row r="39" hidden="1" outlineLevel="1">
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Rent paid — August</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="n">
-        <v>-650</v>
-      </c>
-    </row>
-    <row r="40" hidden="1" outlineLevel="1">
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>New repair tool</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="n">
-        <v>-400</v>
-      </c>
-    </row>
-    <row r="41" hidden="1" outlineLevel="1">
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Credit card paid off</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="n">
-        <v>-2030</v>
-      </c>
-    </row>
-    <row r="42" hidden="1" outlineLevel="1">
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Money taken out for personal use</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="n">
         <v>-600</v>
       </c>
     </row>
-    <row r="43" collapsed="1">
-      <c r="B43" s="16" t="inlineStr">
+    <row r="32" collapsed="1">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>Balance, August 31, 2026</t>
         </is>
       </c>
-      <c r="C43" s="17" t="n"/>
-      <c r="D43" s="13">
-        <f>SUBTOTAL(9,D3:D42)</f>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="13">
+        <f>SUBTOTAL(9,D3:D31)</f>
         <v>620</v>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="6" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="7" t="n"/>
+      <c r="D33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="7" t="n"/>
+      <c r="D34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Right of Use</t>
         </is>
       </c>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="11" t="n"/>
+    </row>
+    <row r="36" hidden="1" outlineLevel="1">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Company received at formation (June 1)</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="37" collapsed="1">
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>Balance, August 31, 2026</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="n"/>
+      <c r="D37" s="13">
+        <f>SUM(D36:D36)</f>
+        <v>650</v>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="7" t="n"/>
+      <c r="D38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Parts</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Company received at formation (June 1)</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Chains ×10 (June)</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>11-spd cassettes ×4 (June)</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="43" hidden="1" outlineLevel="1">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Brake pad sets ×12 (June)</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="n"/>
+      <c r="D43" s="4" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="44" hidden="1" outlineLevel="1">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Cables + housing (assorted) (June)</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" hidden="1" outlineLevel="1">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Tubes ×10 (June)</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Chainrings + jockey wheels (July)</t>
+        </is>
+      </c>
       <c r="C46" s="11" t="n"/>
-      <c r="D46" s="11" t="n"/>
+      <c r="D46" s="4" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="47" hidden="1" outlineLevel="1">
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Last month's rent, paid in advance (on deposit)</t>
+          <t>Bottom brackets ×3 (July)</t>
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="48" collapsed="1">
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>Balance, August 31, 2026</t>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="48" hidden="1" outlineLevel="1">
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Shift cables + housing (July)</t>
         </is>
       </c>
       <c r="C48" s="17" t="n"/>
-      <c r="D48" s="13">
-        <f>D47</f>
-        <v>650</v>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Parts</t>
+      <c r="D48" s="4" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="49" hidden="1" outlineLevel="1">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Tubeless sealant + valves (July)</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1">
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Spokes + nipples (July)</t>
         </is>
       </c>
       <c r="C50" s="11" t="n"/>
-      <c r="D50" s="11" t="n"/>
+      <c r="D50" s="4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="51" hidden="1" outlineLevel="1">
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Chains</t>
+          <t>Tires ×4 (August)</t>
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="52" hidden="1" outlineLevel="1">
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Brake pads</t>
+          <t>Brake pads (assorted) (August)</t>
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
     </row>
     <row r="53" hidden="1" outlineLevel="1">
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Derailleur cables</t>
+          <t>Cables + housing (August)</t>
         </is>
       </c>
       <c r="D53" s="4" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" hidden="1" outlineLevel="1">
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Cassettes</t>
+          <t>Tubes ×8 (August)</t>
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55" hidden="1" outlineLevel="1">
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Bottom brackets</t>
+          <t>Small parts (bolts, tape) (August)</t>
         </is>
       </c>
       <c r="D55" s="4" t="n">
@@ -1039,632 +1055,356 @@
     <row r="56" hidden="1" outlineLevel="1">
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Spokes</t>
+          <t>Parts used — Dana R.</t>
         </is>
       </c>
       <c r="D56" s="4" t="n">
-        <v>20</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="57" hidden="1" outlineLevel="1">
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Tubes</t>
+          <t>Parts used — Priya S.</t>
         </is>
       </c>
       <c r="D57" s="4" t="n">
-        <v>10</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="58" hidden="1" outlineLevel="1">
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Chains ×10 (June)</t>
+          <t>Parts used — Liam O.</t>
         </is>
       </c>
       <c r="D58" s="4" t="n">
-        <v>150</v>
+        <v>-95</v>
       </c>
     </row>
     <row r="59" hidden="1" outlineLevel="1">
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>11-spd cassettes ×4 (June)</t>
+          <t>Parts used — Jamal W.</t>
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>160</v>
+        <v>-60</v>
       </c>
     </row>
     <row r="60" hidden="1" outlineLevel="1">
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Brake pad sets ×12 (June)</t>
+          <t>Parts used — Erin K.</t>
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>90</v>
+        <v>-40</v>
       </c>
     </row>
     <row r="61" hidden="1" outlineLevel="1">
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Cables + housing (assorted) (June)</t>
+          <t>Parts used — Noah B.</t>
         </is>
       </c>
       <c r="D61" s="4" t="n">
-        <v>60</v>
+        <v>-65</v>
       </c>
     </row>
     <row r="62" hidden="1" outlineLevel="1">
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Tubes ×10 (June)</t>
+          <t>Parts used — Grace L.</t>
         </is>
       </c>
       <c r="D62" s="4" t="n">
-        <v>40</v>
+        <v>-35</v>
       </c>
     </row>
     <row r="63" hidden="1" outlineLevel="1">
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Chainrings + jockey wheels (July)</t>
+          <t>Parts used — Theo H.</t>
         </is>
       </c>
       <c r="D63" s="4" t="n">
-        <v>120</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="64" hidden="1" outlineLevel="1">
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Bottom brackets ×3 (July)</t>
+          <t>Parts used — Maya P.</t>
         </is>
       </c>
       <c r="D64" s="4" t="n">
-        <v>105</v>
+        <v>-125</v>
       </c>
     </row>
     <row r="65" hidden="1" outlineLevel="1">
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Shift cables + housing (July)</t>
+          <t>Parts used — Owen C.</t>
         </is>
       </c>
       <c r="D65" s="4" t="n">
-        <v>75</v>
+        <v>-55</v>
       </c>
     </row>
     <row r="66" hidden="1" outlineLevel="1">
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Tubeless sealant + valves (July)</t>
+          <t>Parts used — Ava D.</t>
         </is>
       </c>
       <c r="D66" s="4" t="n">
-        <v>60</v>
+        <v>-45</v>
       </c>
     </row>
     <row r="67" hidden="1" outlineLevel="1">
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Spokes + nipples (July)</t>
+          <t>Parts used — Leo F.</t>
         </is>
       </c>
       <c r="D67" s="4" t="n">
-        <v>40</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="68" hidden="1" outlineLevel="1">
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Tires ×4 (August)</t>
+          <t>Parts used — Nina V.</t>
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>130</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="69" hidden="1" outlineLevel="1">
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Brake pads (assorted) (August)</t>
+          <t>Parts used — Caleb G.</t>
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>70</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="70" hidden="1" outlineLevel="1">
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Cables + housing (August)</t>
+          <t>Parts used — Ruth A.</t>
         </is>
       </c>
       <c r="D70" s="4" t="n">
-        <v>50</v>
+        <v>-129</v>
       </c>
     </row>
     <row r="71" hidden="1" outlineLevel="1">
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Tubes ×8 (August)</t>
+          <t>Parts used — Sam Q.</t>
         </is>
       </c>
       <c r="D71" s="4" t="n">
-        <v>30</v>
+        <v>-70</v>
       </c>
     </row>
     <row r="72" hidden="1" outlineLevel="1">
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Small parts (bolts, tape) (August)</t>
+          <t>Parts used — Westville Bike Share</t>
         </is>
       </c>
       <c r="D72" s="4" t="n">
-        <v>20</v>
+        <v>-105</v>
       </c>
     </row>
     <row r="73" hidden="1" outlineLevel="1">
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Parts used — Dana R.</t>
+          <t>Parts used — Ridgeline Trail Crew</t>
         </is>
       </c>
       <c r="D73" s="4" t="n">
-        <v>-10</v>
+        <v>-75</v>
       </c>
     </row>
     <row r="74" hidden="1" outlineLevel="1">
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Parts used — Priya S.</t>
+          <t>Parts used — J. Smith</t>
         </is>
       </c>
       <c r="D74" s="4" t="n">
-        <v>-25</v>
-      </c>
-    </row>
-    <row r="75" hidden="1" outlineLevel="1">
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Liam O.</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="n">
-        <v>-95</v>
-      </c>
-    </row>
-    <row r="76" hidden="1" outlineLevel="1">
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Jamal W.</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="n">
-        <v>-60</v>
-      </c>
-    </row>
-    <row r="77" hidden="1" outlineLevel="1">
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Erin K.</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="n">
-        <v>-40</v>
-      </c>
+        <v>-36</v>
+      </c>
+    </row>
+    <row r="75" collapsed="1">
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>Balance, August 31, 2026</t>
+        </is>
+      </c>
+      <c r="C75" s="17" t="n"/>
+      <c r="D75" s="13">
+        <f>SUBTOTAL(9,D40:D74)</f>
+        <v>200</v>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="3" t="n"/>
+      <c r="D76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Tools &amp; Repair Equipment</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="n"/>
+      <c r="D77" s="11" t="n"/>
     </row>
     <row r="78" hidden="1" outlineLevel="1">
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Parts used — Noah B.</t>
+          <t>Company received at formation (June 1)</t>
         </is>
       </c>
       <c r="D78" s="4" t="n">
-        <v>-65</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="79" hidden="1" outlineLevel="1">
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Parts used — Grace L.</t>
+          <t>New repair tool bought this season</t>
         </is>
       </c>
       <c r="D79" s="4" t="n">
-        <v>-35</v>
-      </c>
-    </row>
-    <row r="80" hidden="1" outlineLevel="1">
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Theo H.</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="n">
-        <v>-25</v>
-      </c>
-    </row>
-    <row r="81" hidden="1" outlineLevel="1">
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Maya P.</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="n">
-        <v>-125</v>
-      </c>
-    </row>
-    <row r="82" hidden="1" outlineLevel="1">
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Owen C.</t>
-        </is>
-      </c>
-      <c r="D82" s="4" t="n">
-        <v>-55</v>
-      </c>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="80" collapsed="1">
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>Balance, August 31, 2026</t>
+        </is>
+      </c>
+      <c r="C80" s="17" t="n"/>
+      <c r="D80" s="13">
+        <f>SUBTOTAL(9,D78:D79)</f>
+        <v>1600</v>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="3" t="n"/>
+      <c r="D81" s="4" t="n"/>
+    </row>
+    <row r="82">
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Fixtures</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="n"/>
+      <c r="D82" s="11" t="n"/>
     </row>
     <row r="83" hidden="1" outlineLevel="1">
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Parts used — Ava D.</t>
+          <t>Company received at formation (June 1)</t>
         </is>
       </c>
       <c r="D83" s="4" t="n">
-        <v>-45</v>
-      </c>
-    </row>
-    <row r="84" hidden="1" outlineLevel="1">
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Leo F.</t>
-        </is>
-      </c>
-      <c r="D84" s="4" t="n">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="85" hidden="1" outlineLevel="1">
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Nina V.</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="n">
-        <v>-80</v>
-      </c>
-    </row>
-    <row r="86" hidden="1" outlineLevel="1">
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Caleb G.</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="n">
-        <v>-25</v>
-      </c>
+        <v>750</v>
+      </c>
+    </row>
+    <row r="84" collapsed="1">
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>Balance, August 31, 2026</t>
+        </is>
+      </c>
+      <c r="C84" s="17" t="n"/>
+      <c r="D84" s="13">
+        <f>SUM(D83:D83)</f>
+        <v>750</v>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="3" t="n"/>
+      <c r="D85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="n"/>
+      <c r="D86" s="11" t="n"/>
     </row>
     <row r="87" hidden="1" outlineLevel="1">
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Parts used — Ruth A.</t>
+          <t>Company received at formation (June 1)</t>
         </is>
       </c>
       <c r="D87" s="4" t="n">
-        <v>-129</v>
-      </c>
-    </row>
-    <row r="88" hidden="1" outlineLevel="1">
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Sam Q.</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="n">
-        <v>-70</v>
-      </c>
-    </row>
-    <row r="89" hidden="1" outlineLevel="1">
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Westville Bike Share</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="n">
-        <v>-105</v>
-      </c>
-    </row>
-    <row r="90" hidden="1" outlineLevel="1">
-      <c r="B90" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — Ridgeline Trail Crew</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="n">
-        <v>-75</v>
-      </c>
-    </row>
-    <row r="91" hidden="1" outlineLevel="1">
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>Parts used — J. Smith</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="n">
-        <v>-36</v>
-      </c>
-    </row>
-    <row r="92" collapsed="1">
-      <c r="B92" s="16" t="inlineStr">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="88" collapsed="1">
+      <c r="B88" s="16" t="inlineStr">
         <is>
           <t>Balance, August 31, 2026</t>
         </is>
       </c>
-      <c r="C92" s="17" t="n"/>
-      <c r="D92" s="13">
-        <f>SUBTOTAL(9,D51:D91)</f>
-        <v>200</v>
-        <v/>
-      </c>
-    </row>
-    <row r="94">
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>Tools &amp; Repair Equipment</t>
-        </is>
-      </c>
-      <c r="C94" s="11" t="n"/>
-      <c r="D94" s="11" t="n"/>
-    </row>
-    <row r="95" hidden="1" outlineLevel="1">
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t>Repair stand</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="96" hidden="1" outlineLevel="1">
-      <c r="B96" s="3" t="inlineStr">
-        <is>
-          <t>Air compressor</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="n">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="97" hidden="1" outlineLevel="1">
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t>Parts washer</t>
-        </is>
-      </c>
-      <c r="D97" s="4" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="98" hidden="1" outlineLevel="1">
-      <c r="B98" s="3" t="inlineStr">
-        <is>
-          <t>Wheel-truing stand</t>
-        </is>
-      </c>
-      <c r="D98" s="4" t="n">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="99" hidden="1" outlineLevel="1">
-      <c r="B99" s="3" t="inlineStr">
-        <is>
-          <t>Cone wrench set</t>
-        </is>
-      </c>
-      <c r="D99" s="4" t="n">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="100" hidden="1" outlineLevel="1">
-      <c r="B100" s="3" t="inlineStr">
-        <is>
-          <t>Torque wrench</t>
-        </is>
-      </c>
-      <c r="D100" s="4" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="101" hidden="1" outlineLevel="1">
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>Hex/Allen set</t>
-        </is>
-      </c>
-      <c r="D101" s="4" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="102" hidden="1" outlineLevel="1">
-      <c r="B102" s="3" t="inlineStr">
-        <is>
-          <t>Cable cutters</t>
-        </is>
-      </c>
-      <c r="D102" s="4" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="103" hidden="1" outlineLevel="1">
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>Chain breaker</t>
-        </is>
-      </c>
-      <c r="D103" s="4" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="104" hidden="1" outlineLevel="1">
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t>Tire levers</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="105" hidden="1" outlineLevel="1">
-      <c r="B105" s="3" t="inlineStr">
-        <is>
-          <t>Bench grinder</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="106" hidden="1" outlineLevel="1">
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>Headset press</t>
-        </is>
-      </c>
-      <c r="D106" s="4" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="107" hidden="1" outlineLevel="1">
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>Shop vacuum</t>
-        </is>
-      </c>
-      <c r="D107" s="4" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="108" hidden="1" outlineLevel="1">
-      <c r="B108" s="3" t="inlineStr">
-        <is>
-          <t>New repair tool bought this season</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="109" collapsed="1">
-      <c r="B109" s="16" t="inlineStr">
-        <is>
-          <t>Balance, August 31, 2026</t>
-        </is>
-      </c>
-      <c r="C109" s="17" t="n"/>
-      <c r="D109" s="13">
-        <f>SUBTOTAL(9,D95:D108)</f>
-        <v>1600</v>
-        <v/>
-      </c>
-    </row>
-    <row r="111">
-      <c r="B111" s="6" t="inlineStr">
-        <is>
-          <t>Fixtures</t>
-        </is>
-      </c>
-      <c r="C111" s="11" t="n"/>
-      <c r="D111" s="11" t="n"/>
-    </row>
-    <row r="112" hidden="1" outlineLevel="1">
-      <c r="B112" s="3" t="inlineStr">
-        <is>
-          <t>Desk</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="n">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="113" hidden="1" outlineLevel="1">
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>Shelving units</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="114" hidden="1" outlineLevel="1">
-      <c r="B114" s="3" t="inlineStr">
-        <is>
-          <t>Display rack</t>
-        </is>
-      </c>
-      <c r="D114" s="4" t="n">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="115" hidden="1" outlineLevel="1">
-      <c r="B115" s="3" t="inlineStr">
-        <is>
-          <t>Pegboard + hooks</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="116" collapsed="1">
-      <c r="B116" s="16" t="inlineStr">
-        <is>
-          <t>Balance, August 31, 2026</t>
-        </is>
-      </c>
-      <c r="C116" s="17" t="n"/>
-      <c r="D116" s="13">
-        <f>SUM(D112:D115)</f>
-        <v>750</v>
-        <v/>
-      </c>
-    </row>
-    <row r="118">
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C118" s="11" t="n"/>
-      <c r="D118" s="11" t="n"/>
-    </row>
-    <row r="119" hidden="1" outlineLevel="1">
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t>Laptop (from home)</t>
-        </is>
-      </c>
-      <c r="D119" s="4" t="n">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="120" collapsed="1">
-      <c r="B120" s="16" t="inlineStr">
-        <is>
-          <t>Balance, August 31, 2026</t>
-        </is>
-      </c>
-      <c r="C120" s="17" t="n"/>
-      <c r="D120" s="13">
-        <f>SUM(D119)</f>
+      <c r="C88" s="17" t="n"/>
+      <c r="D88" s="13">
+        <f>SUM(D87:D87)</f>
         <v>610</v>
         <v/>
       </c>
     </row>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1677,7 +1417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D15"/>
+  <dimension ref="B1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1702,77 +1442,73 @@
       <c r="C2" s="11" t="n"/>
       <c r="D2" s="11" t="n"/>
     </row>
-    <row r="3" outlineLevel="1">
+    <row r="3" hidden="1" outlineLevel="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Charged — hand tools</t>
+          <t>Company assumed the claim at formation (June 1)</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="4" outlineLevel="1">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="4" hidden="1" outlineLevel="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Charged — air compressor</t>
+          <t>Paid off in full this season</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="5" outlineLevel="1">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Charged — parts washer</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" outlineLevel="1">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Charged — wheel-truing stand</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="7" outlineLevel="1">
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Charged — fixtures</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="8" outlineLevel="1">
+        <v>-2030</v>
+      </c>
+    </row>
+    <row r="5" collapsed="1">
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Balance, August 31, 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="13">
+        <f>SUM(D3:D4)</f>
+        <v>0</v>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="n"/>
+      <c r="D6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Customer Deposit</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+    </row>
+    <row r="8" hidden="1" outlineLevel="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Charged — parts (QBP order)</t>
+          <t>Company assumed the claim at formation (June 1)</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="9" outlineLevel="1">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="9" hidden="1" outlineLevel="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Paid off in full this season</t>
+          <t>Built and delivered Smith's frame — no longer owed</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>-2030</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>-220</v>
+      </c>
+    </row>
+    <row r="10" collapsed="1">
       <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Balance, August 31, 2026</t>
@@ -1780,53 +1516,16 @@
       </c>
       <c r="C10" s="17" t="n"/>
       <c r="D10" s="13">
-        <f>SUM(D3:D9)</f>
+        <f>SUM(D8:D9)</f>
         <v>0</v>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Customer Deposit</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-    </row>
-    <row r="13" outlineLevel="1">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Smith's advance for a custom frame</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="14" outlineLevel="1">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Built and delivered Smith's frame — no longer owed</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>-220</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>Balance, August 31, 2026</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="13">
-        <f>SUM(D13:D14)</f>
-        <v>0</v>
-        <v/>
-      </c>
-    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Wheel truing stand replaces 'New repair tool' (Rick's ruling 2026-08-08) + June-1 canon label repair
The $400 season purchase is now a wheel truing stand across all 13 source
workbooks; regenerated bike-repair-statement-steps.generated.js. Also repairs
a source-of-truth break found tonight: 20 cells still carried 'Company
received at formation (June 1)' where the deployed generated file had been
carrying the June-1 canon 'additional contribution (Section 10)' — the
overnight 2026-08-08 sweep updated the generated file without landing the
label in the workbooks. Sources now agree with canon; formula caches
verified preserved (261/261).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
+++ b/Bike-Repair-Source-Workbooks/Bike-Repair-Beg-Module-3.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D88"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -535,7 +535,7 @@
     <row r="3" hidden="1" outlineLevel="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Company received at formation (June 1)</t>
+          <t>additional contribution (Section 10)</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
@@ -795,7 +795,7 @@
     <row r="29" hidden="1" outlineLevel="1">
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>New repair tool</t>
+          <t>Wheel truing stand</t>
         </is>
       </c>
       <c r="D29" s="4" t="n">
@@ -832,7 +832,6 @@
       <c r="D32" s="13">
         <f>SUBTOTAL(9,D3:D31)</f>
         <v>620</v>
-        <v/>
       </c>
     </row>
     <row r="33">
@@ -872,7 +871,6 @@
       <c r="D37" s="13">
         <f>SUM(D36:D36)</f>
         <v>650</v>
-        <v/>
       </c>
     </row>
     <row r="38">
@@ -1252,7 +1250,6 @@
       <c r="D75" s="13">
         <f>SUBTOTAL(9,D40:D74)</f>
         <v>200</v>
-        <v/>
       </c>
     </row>
     <row r="76">
@@ -1281,7 +1278,7 @@
     <row r="79" hidden="1" outlineLevel="1">
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>New repair tool bought this season</t>
+          <t>Wheel truing stand bought this season</t>
         </is>
       </c>
       <c r="D79" s="4" t="n">
@@ -1298,7 +1295,6 @@
       <c r="D80" s="13">
         <f>SUBTOTAL(9,D78:D79)</f>
         <v>1600</v>
-        <v/>
       </c>
     </row>
     <row r="81">
@@ -1334,7 +1330,6 @@
       <c r="D84" s="13">
         <f>SUM(D83:D83)</f>
         <v>750</v>
-        <v/>
       </c>
     </row>
     <row r="85">
@@ -1370,41 +1365,8 @@
       <c r="D88" s="13">
         <f>SUM(D87:D87)</f>
         <v>610</v>
-        <v/>
-      </c>
-    </row>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1417,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1472,7 +1434,6 @@
       <c r="D5" s="13">
         <f>SUM(D3:D4)</f>
         <v>0</v>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -1518,14 +1479,8 @@
       <c r="D10" s="13">
         <f>SUM(D8:D9)</f>
         <v>0</v>
-        <v/>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1538,7 +1493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D60"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1566,7 +1521,7 @@
     <row r="3" hidden="1" outlineLevel="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Cash — Company received at formation (June 1)</t>
+          <t>Cash — additional contribution (Section 10)</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
@@ -1655,7 +1610,6 @@
       <c r="D11" s="13">
         <f>SUM(D3:D10)</f>
         <v>2460</v>
-        <v/>
       </c>
     </row>
     <row r="12">
@@ -2101,7 +2055,6 @@
       <c r="D56" s="13">
         <f>SUM(D14:D55)</f>
         <v>2570</v>
-        <v/>
       </c>
     </row>
     <row r="57">
@@ -2137,7 +2090,6 @@
       <c r="D60" s="13">
         <f>SUM(D59:D59)</f>
         <v>-600</v>
-        <v/>
       </c>
     </row>
     <row r="64" outlineLevel="1"/>
@@ -2153,7 +2105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>

</xml_diff>